<commit_message>
Fix methodology sheet RTL formatting and update all 9 stock prices
Formatting fix:
- Added readingOrder=2 to all cells in methodology sheet to force RTL
  rendering — resolves mixed Arabic/English alignment issue in Excel

Price updates (closing prices May 2026):
- الراجحي  1120:  69.10 → 66.60  (post bonus-share adjustment 4B→6B)
- الإنماء  1150:  27.50 → 23.53  (user confirmed)
- STC       7010:  42.00 → 43.54  (Apr 30 close)
- سال       4263: 185.00 → 164.10 (Apr 29 close)
- المواساة  4002:  67.00 → 59.10  (Mar 2026)
- بدجت     4260:  38.00 → 75.90  (confirmed — stock nearly doubled)
- اكسترا   4003:  95.00 → 81.90  (Apr 2026)
- المتقدمة 2330:  48.00 → 30.00  (Dec 2025 — latest available)
- بنيان ريت 4340: 10.20 →  9.25  (Mar 2026)

All price changes flow through to P/E, P/B, upside%, and safety margin
calculations across all valuation and overview sheets.

https://claude.ai/code/session_01TsvCZbyBaMSGgSHhDFZ22w
</commit_message>
<xml_diff>
--- a/saudi-investment-analysis/Saudi_Portfolio_Analysis_2026.xlsx
+++ b/saudi-investment-analysis/Saudi_Portfolio_Analysis_2026.xlsx
@@ -579,61 +579,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="261">
+  <cellXfs count="255">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -851,7 +851,7 @@
     <xf numFmtId="0" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -881,7 +881,7 @@
     <xf numFmtId="0" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -932,7 +932,7 @@
     <xf numFmtId="164" fontId="24" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -959,7 +959,7 @@
     <xf numFmtId="164" fontId="24" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -980,16 +980,13 @@
     <xf numFmtId="4" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1016,7 +1013,7 @@
     <xf numFmtId="164" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1051,6 +1048,9 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1077,15 +1077,6 @@
     <xf numFmtId="0" fontId="32" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="33" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1111,7 +1102,7 @@
     <xf numFmtId="4" fontId="33" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="38" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1126,23 +1117,17 @@
     <xf numFmtId="0" fontId="4" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="33" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="30" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="30" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1195,17 +1180,14 @@
     <xf numFmtId="0" fontId="4" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="33" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="30" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="30" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2109,132 +2091,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>42</v>
+      <c r="B3" s="244" t="n">
+        <v>43.54</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>50000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>14.2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>3.82</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>5.2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>26.9</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>تراكم بقوة</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -2261,78 +2243,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>63000</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>67000</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>71800</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>75893</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>11100</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>12200</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>13300</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>24689</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>18000</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>20000</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>22000</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>24500</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: البنية الرقمية الوطنية + 5G + STC Pay + حلول سحابة للقطاع الحكومي</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: CAPEX مرتفع · ملكية حكومية قد تؤثر على قرارات التوزيع · منافسة موبايلي/زين</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: ⚠ ربح 2024 (24.7B) يشمل بيع TAWAL (13.97B غير متكرر) → الربح الجاري ≈ 10.7B ريال</t>
         </is>
@@ -2375,132 +2357,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>185</v>
+      <c r="B3" s="244" t="n">
+        <v>164.1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>80</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>22.4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>6.4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>1.8</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>30.5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>مراقبة / تراكم تدريجي</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -2527,78 +2509,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>900</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>1100</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>1452</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>1630</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>320</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>450</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>511</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>661</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>400</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>550</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>680</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>820</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: مطار الملك سلمان الدولي + نمو الشحن الجوي + خدمات الخطوط السعودية</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: تركيز عملاء عالٍ · IPO تقييم مرتفع · بيانات تاريخية قصيرة · تذبذب الأسعار</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: IPO حديث (2022) - بيانات تاريخية محدودة | ✅ إيرادات 2024: 1.63B ريال (تحقق)</t>
         </is>
@@ -2641,132 +2623,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>67</v>
+      <c r="B3" s="244" t="n">
+        <v>59.1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>2000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>20.7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>3.35</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>17.3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>احتفاظ / تراكم عند الضعف</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -2793,78 +2775,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>2050</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>2400</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>2706</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>2879</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>520</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>680</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>658</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>646</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>650</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>820</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>800</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>780</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: خصخصة الصحة + التأمين الإلزامي + السياحة الطبية + توسع في المدينة</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: تراجع هامش الربح · شح الكوادر الطبية · تنافسية القطاع الخاص المتنامية</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: توزيع سنوي ثابت منذ الإدراج</t>
         </is>
@@ -2907,132 +2889,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>38</v>
+      <c r="B3" s="244" t="n">
+        <v>75.90000000000001</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>12.2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>3.8</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>17.4</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>متوسط-مرتفع</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>مراقبة - انتظار توضيح Q1 2026</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -3059,78 +3041,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>1200</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>1500</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>1750</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>1980</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>185</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>240</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>277</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>312</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>380</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>460</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>510</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>550</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: السياحة + الفعاليات والترفيه + تأجير أسطول NEOM + نمو المطارات</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: ⚠ تراجع ربح Q1 2026 بـ58% · رأس مال مكثف للأسطول · منافسة منصات المشاركة</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: ⚠ انخفاض أرباح Q1 2026 بنسبة 58% - يستوجب مراقبة</t>
         </is>
@@ -3173,132 +3155,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>95</v>
+      <c r="B3" s="244" t="n">
+        <v>81.90000000000001</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>800</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>80</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>14.4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>5.3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>30.1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>تراكم</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -3325,78 +3307,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>4500</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>5200</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>5800</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>6781</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>280</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>340</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>390</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>534</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>350</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>430</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>500</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>620</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: نمو الإنفاق الاستهلاكي + التحول الرقمي + تراخيص جديدة + توسع جغرافي</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: منافسة أمازون.sa ونون · ضغط هوامش التجزئة · التحدي الرقمي</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: ✅ توزيع استثنائي أغسطس 2024: 5 ريال/سهم من الاحتياطيات | ربح FY2024: 534.5M ريال</t>
         </is>
@@ -3439,128 +3421,128 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>48</v>
+      <c r="B3" s="244" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>1250</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n"/>
+      <c r="B6" s="246" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n"/>
+      <c r="B9" s="244" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>مرتفع</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>مضاربة / وزن محدود</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -3587,78 +3569,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>2100</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>2400</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>1900</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>1700</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>380</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>320</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>85</v>
       </c>
-      <c r="E17" s="260" t="n">
+      <c r="E17" s="254" t="n">
         <v>-259</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>450</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>380</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>180</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: تحويل البلاستيك للمواد الإنشائية (NEOM) + طاقة انتاجية جديدة + تنويع المنتجات</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: ⚠ دورية البتروكيماويات · خسارة 2024 · أسعار البروبيلين العالمية · منافسة صينية</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: ⚠ لا توزيعات 2023-2024 بسبب الخسارة | العودة للربحية Q1 2025</t>
         </is>
@@ -3701,132 +3683,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>10.2</v>
+      <c r="B3" s="244" t="n">
+        <v>9.25</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>1630</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>163</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>14.1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>1.03</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>7.5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>7.3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>احتفاظ للدخل</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -3853,78 +3835,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>140</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>155</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>170</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>190</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>85</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>95</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>105</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>118</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>90</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>100</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>115</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: نمو القطاع العقاري + الطلب السياحي + نمو الإيجارات التجارية</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: حساسية أسعار الفائدة · جودة المستأجرين · إعادة التقييم العقاري · تركيز الأصول</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: توزيع نصف سنوي إلزامي ≥90% من الدخل الصافي</t>
         </is>
@@ -4083,7 +4065,7 @@
         </is>
       </c>
       <c r="E4" s="25" t="n">
-        <v>69.09999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F4" s="26" t="n">
         <v>14</v>
@@ -4139,7 +4121,7 @@
         </is>
       </c>
       <c r="E5" s="31" t="n">
-        <v>27.5</v>
+        <v>23.53</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>9.4</v>
@@ -4195,7 +4177,7 @@
         </is>
       </c>
       <c r="E6" s="25" t="n">
-        <v>42</v>
+        <v>43.54</v>
       </c>
       <c r="F6" s="26" t="n">
         <v>14.2</v>
@@ -4251,7 +4233,7 @@
         </is>
       </c>
       <c r="E7" s="31" t="n">
-        <v>185</v>
+        <v>164.1</v>
       </c>
       <c r="F7" s="32" t="n">
         <v>22.4</v>
@@ -4307,7 +4289,7 @@
         </is>
       </c>
       <c r="E8" s="38" t="n">
-        <v>67</v>
+        <v>59.1</v>
       </c>
       <c r="F8" s="39" t="n">
         <v>20.7</v>
@@ -4363,7 +4345,7 @@
         </is>
       </c>
       <c r="E9" s="31" t="n">
-        <v>38</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F9" s="32" t="n">
         <v>12.2</v>
@@ -4419,7 +4401,7 @@
         </is>
       </c>
       <c r="E10" s="38" t="n">
-        <v>95</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="F10" s="39" t="n">
         <v>14.4</v>
@@ -4475,7 +4457,7 @@
         </is>
       </c>
       <c r="E11" s="25" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="F11" s="24" t="inlineStr">
         <is>
@@ -4537,7 +4519,7 @@
         </is>
       </c>
       <c r="E12" s="38" t="n">
-        <v>10.2</v>
+        <v>9.25</v>
       </c>
       <c r="F12" s="39" t="n">
         <v>14.1</v>
@@ -4616,7 +4598,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  الراجحي (1120) — مصرفي  ⚠ منح سهم لكل سهمين في H2 2025 → سترتفع الأسهم إلى 6,000M</t>
+          <t xml:space="preserve">  الراجحي (1120) — مصرفي  ✅ سعر مُعدَّل بعد المنح (1 سهم / 2) → الأسهم ارتفعت من 4B إلى 6B</t>
         </is>
       </c>
     </row>
@@ -9043,7 +9025,7 @@
         </is>
       </c>
       <c r="B4" s="83" t="n">
-        <v>69.09999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="C4" s="84" t="n">
         <v>14</v>
@@ -9058,7 +9040,7 @@
         <v>1.46</v>
       </c>
       <c r="G4" s="85" t="n">
-        <v>8.1</v>
+        <v>7.8</v>
       </c>
       <c r="H4" s="88" t="n">
         <v>83</v>
@@ -9082,7 +9064,7 @@
       </c>
       <c r="N4" s="91" t="inlineStr">
         <is>
-          <t>+7.4%</t>
+          <t>+11.4%</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9075,7 @@
         </is>
       </c>
       <c r="B5" s="93" t="n">
-        <v>27.5</v>
+        <v>23.53</v>
       </c>
       <c r="C5" s="94" t="n">
         <v>9.4</v>
@@ -9108,7 +9090,7 @@
         <v>0.32</v>
       </c>
       <c r="G5" s="95" t="n">
-        <v>5.4</v>
+        <v>4.6</v>
       </c>
       <c r="H5" s="98" t="n">
         <v>35</v>
@@ -9132,7 +9114,7 @@
       </c>
       <c r="N5" s="101" t="inlineStr">
         <is>
-          <t>+4.7%</t>
+          <t>+22.4%</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9125,7 @@
         </is>
       </c>
       <c r="B6" s="103" t="n">
-        <v>42</v>
+        <v>43.54</v>
       </c>
       <c r="C6" s="104" t="n">
         <v>14.2</v>
@@ -9158,7 +9140,7 @@
         <v>0.47</v>
       </c>
       <c r="G6" s="105" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="H6" s="108" t="n">
         <v>51</v>
@@ -9180,7 +9162,7 @@
       </c>
       <c r="N6" s="109" t="inlineStr">
         <is>
-          <t>+16.9%</t>
+          <t>+12.8%</t>
         </is>
       </c>
     </row>
@@ -9191,7 +9173,7 @@
         </is>
       </c>
       <c r="B7" s="111" t="n">
-        <v>185</v>
+        <v>164.1</v>
       </c>
       <c r="C7" s="112" t="n">
         <v>22.4</v>
@@ -9206,7 +9188,7 @@
         <v>0.82</v>
       </c>
       <c r="G7" s="113" t="n">
-        <v>9.1</v>
+        <v>8.1</v>
       </c>
       <c r="H7" s="116" t="n">
         <v>220</v>
@@ -9223,12 +9205,12 @@
       <c r="L7" s="117" t="n">
         <v>137.8</v>
       </c>
-      <c r="M7" s="117" t="n">
+      <c r="M7" s="116" t="n">
         <v>178.4</v>
       </c>
       <c r="N7" s="118" t="inlineStr">
         <is>
-          <t>-2.1%</t>
+          <t>+10.4%</t>
         </is>
       </c>
     </row>
@@ -9239,7 +9221,7 @@
         </is>
       </c>
       <c r="B8" s="120" t="n">
-        <v>67</v>
+        <v>59.1</v>
       </c>
       <c r="C8" s="121" t="n">
         <v>20.7</v>
@@ -9254,7 +9236,7 @@
         <v>2.76</v>
       </c>
       <c r="G8" s="122" t="n">
-        <v>4.7</v>
+        <v>4.1</v>
       </c>
       <c r="H8" s="125" t="n">
         <v>74</v>
@@ -9268,7 +9250,7 @@
       <c r="K8" s="126" t="n">
         <v>52.1</v>
       </c>
-      <c r="L8" s="126" t="n">
+      <c r="L8" s="125" t="n">
         <v>61.2</v>
       </c>
       <c r="M8" s="125" t="n">
@@ -9276,7 +9258,7 @@
       </c>
       <c r="N8" s="127" t="inlineStr">
         <is>
-          <t>+0.7%</t>
+          <t>+14.2%</t>
         </is>
       </c>
     </row>
@@ -9287,7 +9269,7 @@
         </is>
       </c>
       <c r="B9" s="129" t="n">
-        <v>38</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="C9" s="130" t="n">
         <v>12.2</v>
@@ -9302,12 +9284,12 @@
         <v>0.64</v>
       </c>
       <c r="G9" s="131" t="n">
-        <v>1.9</v>
+        <v>3.8</v>
       </c>
       <c r="H9" s="134" t="n">
         <v>46</v>
       </c>
-      <c r="I9" s="135" t="n">
+      <c r="I9" s="134" t="n">
         <v>38</v>
       </c>
       <c r="J9" s="134" t="n">
@@ -9319,12 +9301,12 @@
       <c r="L9" s="134" t="n">
         <v>49.3</v>
       </c>
-      <c r="M9" s="134" t="n">
+      <c r="M9" s="135" t="n">
         <v>90.2</v>
       </c>
       <c r="N9" s="136" t="inlineStr">
         <is>
-          <t>+16.1%</t>
+          <t>-41.9%</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9317,7 @@
         </is>
       </c>
       <c r="B10" s="111" t="n">
-        <v>95</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C10" s="112" t="n">
         <v>14.4</v>
@@ -9350,7 +9332,7 @@
         <v>0.6</v>
       </c>
       <c r="G10" s="113" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="H10" s="116" t="n">
         <v>115</v>
@@ -9364,128 +9346,128 @@
       <c r="K10" s="116" t="n">
         <v>106.2</v>
       </c>
-      <c r="L10" s="117" t="n">
+      <c r="L10" s="116" t="n">
         <v>86.8</v>
       </c>
       <c r="M10" s="116" t="n">
         <v>111.7</v>
       </c>
-      <c r="N10" s="137" t="inlineStr">
-        <is>
-          <t>+7.6%</t>
+      <c r="N10" s="118" t="inlineStr">
+        <is>
+          <t>+24.8%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="138" t="inlineStr">
+      <c r="A11" s="137" t="inlineStr">
         <is>
           <t>المتقدمة</t>
         </is>
       </c>
-      <c r="B11" s="139" t="n">
-        <v>48</v>
-      </c>
-      <c r="C11" s="140" t="inlineStr">
+      <c r="B11" s="138" t="n">
+        <v>30</v>
+      </c>
+      <c r="C11" s="139" t="inlineStr">
         <is>
           <t>خسارة</t>
         </is>
       </c>
-      <c r="D11" s="141" t="n">
+      <c r="D11" s="140" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="142" t="n">
+      <c r="E11" s="141" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="143" t="inlineStr">
+      <c r="F11" s="142" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="141" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="H11" s="144" t="n">
+      <c r="G11" s="140" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H11" s="143" t="n">
         <v>60</v>
       </c>
-      <c r="I11" s="143" t="inlineStr">
+      <c r="I11" s="142" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J11" s="144" t="n">
+      <c r="J11" s="143" t="n">
         <v>55</v>
       </c>
-      <c r="K11" s="143" t="inlineStr">
+      <c r="K11" s="142" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="L11" s="145" t="n">
+      <c r="L11" s="144" t="n">
         <v>3.6</v>
       </c>
-      <c r="M11" s="145" t="n">
+      <c r="M11" s="143" t="n">
         <v>38.8</v>
       </c>
-      <c r="N11" s="146" t="inlineStr">
-        <is>
-          <t>-17.7%</t>
+      <c r="N11" s="145" t="inlineStr">
+        <is>
+          <t>+31.7%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="147" t="inlineStr">
+      <c r="A12" s="146" t="inlineStr">
         <is>
           <t>بنيان ريت</t>
         </is>
       </c>
-      <c r="B12" s="148" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="C12" s="149" t="n">
+      <c r="B12" s="147" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="C12" s="148" t="n">
         <v>14.1</v>
       </c>
-      <c r="D12" s="150" t="n">
+      <c r="D12" s="149" t="n">
         <v>1.03</v>
       </c>
-      <c r="E12" s="151" t="n">
+      <c r="E12" s="150" t="n">
         <v>7.5</v>
       </c>
-      <c r="F12" s="152" t="n">
+      <c r="F12" s="151" t="n">
         <v>1.22</v>
       </c>
-      <c r="G12" s="150" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="H12" s="153" t="n">
+      <c r="G12" s="149" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H12" s="152" t="n">
         <v>10.8</v>
       </c>
-      <c r="I12" s="153" t="n">
+      <c r="I12" s="152" t="n">
         <v>11.5</v>
       </c>
-      <c r="J12" s="153" t="n">
+      <c r="J12" s="152" t="n">
         <v>10.5</v>
       </c>
-      <c r="K12" s="153" t="n">
+      <c r="K12" s="152" t="n">
         <v>14.8</v>
       </c>
-      <c r="L12" s="154" t="inlineStr">
+      <c r="L12" s="153" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="M12" s="154" t="inlineStr">
+      <c r="M12" s="153" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="N12" s="155" t="inlineStr">
-        <is>
-          <t>+16.7%</t>
+      <c r="N12" s="154" t="inlineStr">
+        <is>
+          <t>+28.6%</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="156" t="inlineStr">
+      <c r="A14" s="155" t="inlineStr">
         <is>
           <t>منهجية: P/E = متوسط P/E قطاعي × EPS 2024  |  P/B = متوسط P/B قطاعي × القيمة الدفترية  |  DDM = DPS₁/(WACC−g)  |  DCF = Σ FCF/(1+WACC)^t + Terminal (5 سنوات، g_terminal=3%)  |  EV/EBITDA = EBITDA × Benchmark القطاعي ÷ الأسهم  |  PEG = P/E ÷ CAGR%  |  هامش الأمان = (متوسط 5 طرق − السعر) ÷ السعر  |  ⚠ DCF وEV/EBITDA تقديرات مبنية على OCF كـProxy — راجع ورقة منهجية التقييم للتفاصيل</t>
         </is>
@@ -9527,46 +9509,46 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="157" t="inlineStr">
+      <c r="A2" s="156" t="inlineStr">
         <is>
           <t>⚠ ملاحظة: أسعار بيوت الخبرة المسماة محدودة الإتاحة للعموم — البيانات المُتحقق منها تعتمد على إجماع Investing.com/Bloomberg. | ⚠ أهداف بدجت مُحتسبة قبل نتائج Q1 2026 المخيبة للآمال.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="157" t="inlineStr">
         <is>
           <t>الشركة</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="157" t="inlineStr">
         <is>
           <t>الرمز</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="157" t="inlineStr">
         <is>
           <t>السعر الحالي
 (ريال)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="157" t="inlineStr">
         <is>
           <t>بيت الخبرة / المصدر</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="157" t="inlineStr">
         <is>
           <t>السعر المستهدف
 (ريال)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="157" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="157" t="inlineStr">
         <is>
           <t>Upside%</t>
         </is>
@@ -9584,7 +9566,7 @@
         </is>
       </c>
       <c r="C4" s="160" t="n">
-        <v>69.09999999999999</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="D4" s="161" t="inlineStr">
         <is>
@@ -9601,7 +9583,7 @@
       </c>
       <c r="G4" s="164" t="inlineStr">
         <is>
-          <t>+47.6%</t>
+          <t>+53.2%</t>
         </is>
       </c>
     </row>
@@ -9624,7 +9606,7 @@
       </c>
       <c r="G5" s="164" t="inlineStr">
         <is>
-          <t>+36.8%</t>
+          <t>+41.9%</t>
         </is>
       </c>
     </row>
@@ -9647,7 +9629,7 @@
       </c>
       <c r="G6" s="164" t="inlineStr">
         <is>
-          <t>+64.3%</t>
+          <t>+70.4%</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9652,7 @@
       </c>
       <c r="G7" s="164" t="inlineStr">
         <is>
-          <t>+82.3%</t>
+          <t>+89.2%</t>
         </is>
       </c>
     </row>
@@ -9693,7 +9675,7 @@
       </c>
       <c r="G8" s="164" t="inlineStr">
         <is>
-          <t>+43.8%</t>
+          <t>+49.2%</t>
         </is>
       </c>
     </row>
@@ -9716,7 +9698,7 @@
         </is>
       </c>
       <c r="C10" s="160" t="n">
-        <v>27.5</v>
+        <v>23.53</v>
       </c>
       <c r="D10" s="161" t="inlineStr">
         <is>
@@ -9731,9 +9713,9 @@
           <t>شراء (Buy)</t>
         </is>
       </c>
-      <c r="G10" s="167" t="inlineStr">
-        <is>
-          <t>+0.4%</t>
+      <c r="G10" s="164" t="inlineStr">
+        <is>
+          <t>+17.3%</t>
         </is>
       </c>
     </row>
@@ -9756,7 +9738,7 @@
       </c>
       <c r="G11" s="164" t="inlineStr">
         <is>
-          <t>+49.1%</t>
+          <t>+74.2%</t>
         </is>
       </c>
     </row>
@@ -9769,7 +9751,7 @@
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E12" s="168" t="n">
+      <c r="E12" s="162" t="n">
         <v>25</v>
       </c>
       <c r="F12" s="163" t="inlineStr">
@@ -9777,9 +9759,9 @@
           <t>محايد</t>
         </is>
       </c>
-      <c r="G12" s="169" t="inlineStr">
-        <is>
-          <t>-9.1%</t>
+      <c r="G12" s="164" t="inlineStr">
+        <is>
+          <t>+6.2%</t>
         </is>
       </c>
     </row>
@@ -9791,81 +9773,81 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="170" t="inlineStr">
+      <c r="A14" s="167" t="inlineStr">
         <is>
           <t>STC</t>
         </is>
       </c>
-      <c r="B14" s="171" t="inlineStr">
+      <c r="B14" s="168" t="inlineStr">
         <is>
           <t>7010</t>
         </is>
       </c>
-      <c r="C14" s="172" t="n">
-        <v>42</v>
-      </c>
-      <c r="D14" s="173" t="inlineStr">
+      <c r="C14" s="169" t="n">
+        <v>43.54</v>
+      </c>
+      <c r="D14" s="170" t="inlineStr">
         <is>
           <t>إجماع (8 محللين)</t>
         </is>
       </c>
-      <c r="E14" s="174" t="n">
+      <c r="E14" s="171" t="n">
         <v>47.7</v>
       </c>
-      <c r="F14" s="175" t="inlineStr">
+      <c r="F14" s="172" t="inlineStr">
         <is>
           <t>شراء (Buy)</t>
         </is>
       </c>
-      <c r="G14" s="176" t="inlineStr">
-        <is>
-          <t>+13.6%</t>
+      <c r="G14" s="173" t="inlineStr">
+        <is>
+          <t>+9.6%</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="177" t="inlineStr"/>
-      <c r="B15" s="177" t="inlineStr"/>
-      <c r="C15" s="177" t="inlineStr"/>
-      <c r="D15" s="173" t="inlineStr">
+      <c r="A15" s="174" t="inlineStr"/>
+      <c r="B15" s="174" t="inlineStr"/>
+      <c r="C15" s="174" t="inlineStr"/>
+      <c r="D15" s="170" t="inlineStr">
         <is>
           <t>الأعلى (High)</t>
         </is>
       </c>
-      <c r="E15" s="174" t="n">
+      <c r="E15" s="171" t="n">
         <v>55</v>
       </c>
-      <c r="F15" s="175" t="inlineStr">
+      <c r="F15" s="172" t="inlineStr">
         <is>
           <t>شراء قوي</t>
         </is>
       </c>
-      <c r="G15" s="176" t="inlineStr">
-        <is>
-          <t>+31.0%</t>
+      <c r="G15" s="173" t="inlineStr">
+        <is>
+          <t>+26.3%</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="177" t="inlineStr"/>
-      <c r="B16" s="177" t="inlineStr"/>
-      <c r="C16" s="177" t="inlineStr"/>
-      <c r="D16" s="173" t="inlineStr">
+      <c r="A16" s="174" t="inlineStr"/>
+      <c r="B16" s="174" t="inlineStr"/>
+      <c r="C16" s="174" t="inlineStr"/>
+      <c r="D16" s="170" t="inlineStr">
         <is>
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E16" s="178" t="n">
+      <c r="E16" s="175" t="n">
         <v>41.1</v>
       </c>
-      <c r="F16" s="175" t="inlineStr">
+      <c r="F16" s="172" t="inlineStr">
         <is>
           <t>محايد</t>
         </is>
       </c>
-      <c r="G16" s="179" t="inlineStr">
-        <is>
-          <t>-2.1%</t>
+      <c r="G16" s="176" t="inlineStr">
+        <is>
+          <t>-5.6%</t>
         </is>
       </c>
     </row>
@@ -9877,81 +9859,81 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="180" t="inlineStr">
+      <c r="A18" s="177" t="inlineStr">
         <is>
           <t>سال</t>
         </is>
       </c>
-      <c r="B18" s="181" t="inlineStr">
+      <c r="B18" s="178" t="inlineStr">
         <is>
           <t>4263</t>
         </is>
       </c>
-      <c r="C18" s="182" t="n">
-        <v>185</v>
-      </c>
-      <c r="D18" s="183" t="inlineStr">
+      <c r="C18" s="179" t="n">
+        <v>164.1</v>
+      </c>
+      <c r="D18" s="180" t="inlineStr">
         <is>
           <t>إجماع المحللين</t>
         </is>
       </c>
-      <c r="E18" s="184" t="n">
+      <c r="E18" s="181" t="n">
         <v>178.4</v>
       </c>
-      <c r="F18" s="185" t="inlineStr">
+      <c r="F18" s="182" t="inlineStr">
         <is>
           <t>محايد (Neutral)</t>
         </is>
       </c>
-      <c r="G18" s="186" t="inlineStr">
-        <is>
-          <t>-3.6%</t>
+      <c r="G18" s="183" t="inlineStr">
+        <is>
+          <t>+8.7%</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="187" t="inlineStr"/>
-      <c r="B19" s="187" t="inlineStr"/>
-      <c r="C19" s="187" t="inlineStr"/>
-      <c r="D19" s="183" t="inlineStr">
+      <c r="A19" s="184" t="inlineStr"/>
+      <c r="B19" s="184" t="inlineStr"/>
+      <c r="C19" s="184" t="inlineStr"/>
+      <c r="D19" s="180" t="inlineStr">
         <is>
           <t>الأعلى (High)</t>
         </is>
       </c>
-      <c r="E19" s="188" t="n">
+      <c r="E19" s="181" t="n">
         <v>196.1</v>
       </c>
-      <c r="F19" s="185" t="inlineStr">
+      <c r="F19" s="182" t="inlineStr">
         <is>
           <t>شراء</t>
         </is>
       </c>
-      <c r="G19" s="189" t="inlineStr">
-        <is>
-          <t>+6.0%</t>
+      <c r="G19" s="183" t="inlineStr">
+        <is>
+          <t>+19.5%</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="187" t="inlineStr"/>
-      <c r="B20" s="187" t="inlineStr"/>
-      <c r="C20" s="187" t="inlineStr"/>
-      <c r="D20" s="183" t="inlineStr">
+      <c r="A20" s="184" t="inlineStr"/>
+      <c r="B20" s="184" t="inlineStr"/>
+      <c r="C20" s="184" t="inlineStr"/>
+      <c r="D20" s="180" t="inlineStr">
         <is>
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E20" s="184" t="n">
+      <c r="E20" s="181" t="n">
         <v>165</v>
       </c>
-      <c r="F20" s="185" t="inlineStr">
+      <c r="F20" s="182" t="inlineStr">
         <is>
           <t>محايد</t>
         </is>
       </c>
-      <c r="G20" s="190" t="inlineStr">
-        <is>
-          <t>-10.8%</t>
+      <c r="G20" s="185" t="inlineStr">
+        <is>
+          <t>+0.5%</t>
         </is>
       </c>
     </row>
@@ -9963,81 +9945,81 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="191" t="inlineStr">
+      <c r="A22" s="186" t="inlineStr">
         <is>
           <t>المواساة</t>
         </is>
       </c>
-      <c r="B22" s="192" t="inlineStr">
+      <c r="B22" s="187" t="inlineStr">
         <is>
           <t>4002</t>
         </is>
       </c>
-      <c r="C22" s="193" t="n">
-        <v>67</v>
-      </c>
-      <c r="D22" s="194" t="inlineStr">
+      <c r="C22" s="188" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="D22" s="189" t="inlineStr">
         <is>
           <t>إجماع (5+ محللين)</t>
         </is>
       </c>
-      <c r="E22" s="195" t="n">
+      <c r="E22" s="190" t="n">
         <v>91.59999999999999</v>
       </c>
-      <c r="F22" s="196" t="inlineStr">
+      <c r="F22" s="191" t="inlineStr">
         <is>
           <t>شراء (Buy)</t>
         </is>
       </c>
-      <c r="G22" s="197" t="inlineStr">
-        <is>
-          <t>+36.7%</t>
+      <c r="G22" s="192" t="inlineStr">
+        <is>
+          <t>+55.0%</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="198" t="inlineStr"/>
-      <c r="B23" s="198" t="inlineStr"/>
-      <c r="C23" s="198" t="inlineStr"/>
-      <c r="D23" s="194" t="inlineStr">
+      <c r="A23" s="193" t="inlineStr"/>
+      <c r="B23" s="193" t="inlineStr"/>
+      <c r="C23" s="193" t="inlineStr"/>
+      <c r="D23" s="189" t="inlineStr">
         <is>
           <t>الأعلى (High)</t>
         </is>
       </c>
-      <c r="E23" s="195" t="n">
+      <c r="E23" s="190" t="n">
         <v>125</v>
       </c>
-      <c r="F23" s="196" t="inlineStr">
+      <c r="F23" s="191" t="inlineStr">
         <is>
           <t>شراء قوي</t>
         </is>
       </c>
-      <c r="G23" s="197" t="inlineStr">
-        <is>
-          <t>+86.6%</t>
+      <c r="G23" s="192" t="inlineStr">
+        <is>
+          <t>+111.5%</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="198" t="inlineStr"/>
-      <c r="B24" s="198" t="inlineStr"/>
-      <c r="C24" s="198" t="inlineStr"/>
-      <c r="D24" s="194" t="inlineStr">
+      <c r="A24" s="193" t="inlineStr"/>
+      <c r="B24" s="193" t="inlineStr"/>
+      <c r="C24" s="193" t="inlineStr"/>
+      <c r="D24" s="189" t="inlineStr">
         <is>
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E24" s="195" t="n">
+      <c r="E24" s="190" t="n">
         <v>75.5</v>
       </c>
-      <c r="F24" s="196" t="inlineStr">
+      <c r="F24" s="191" t="inlineStr">
         <is>
           <t>محايد</t>
         </is>
       </c>
-      <c r="G24" s="197" t="inlineStr">
-        <is>
-          <t>+12.7%</t>
+      <c r="G24" s="192" t="inlineStr">
+        <is>
+          <t>+27.7%</t>
         </is>
       </c>
     </row>
@@ -10049,81 +10031,81 @@
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="199" t="inlineStr">
+      <c r="A26" s="194" t="inlineStr">
         <is>
           <t>بدجت</t>
         </is>
       </c>
-      <c r="B26" s="200" t="inlineStr">
+      <c r="B26" s="195" t="inlineStr">
         <is>
           <t>4260</t>
         </is>
       </c>
-      <c r="C26" s="201" t="n">
-        <v>38</v>
-      </c>
-      <c r="D26" s="202" t="inlineStr">
+      <c r="C26" s="196" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="D26" s="197" t="inlineStr">
         <is>
           <t>⚠ إجماع (8) — قبل انهيار Q1</t>
         </is>
       </c>
-      <c r="E26" s="203" t="n">
+      <c r="E26" s="198" t="n">
         <v>90.2</v>
       </c>
-      <c r="F26" s="204" t="inlineStr">
+      <c r="F26" s="199" t="inlineStr">
         <is>
           <t>شراء قوي — يستوجب مراجعة</t>
         </is>
       </c>
-      <c r="G26" s="205" t="inlineStr">
-        <is>
-          <t>+137.4%</t>
+      <c r="G26" s="200" t="inlineStr">
+        <is>
+          <t>+18.8%</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="206" t="inlineStr"/>
-      <c r="B27" s="206" t="inlineStr"/>
-      <c r="C27" s="206" t="inlineStr"/>
-      <c r="D27" s="202" t="inlineStr">
+      <c r="A27" s="201" t="inlineStr"/>
+      <c r="B27" s="201" t="inlineStr"/>
+      <c r="C27" s="201" t="inlineStr"/>
+      <c r="D27" s="197" t="inlineStr">
         <is>
           <t>الأعلى (High) — قبل Q1</t>
         </is>
       </c>
-      <c r="E27" s="203" t="n">
+      <c r="E27" s="198" t="n">
         <v>100</v>
       </c>
-      <c r="F27" s="204" t="inlineStr">
+      <c r="F27" s="199" t="inlineStr">
         <is>
           <t>شراء قوي</t>
         </is>
       </c>
-      <c r="G27" s="205" t="inlineStr">
-        <is>
-          <t>+163.2%</t>
+      <c r="G27" s="200" t="inlineStr">
+        <is>
+          <t>+31.8%</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="206" t="inlineStr"/>
-      <c r="B28" s="206" t="inlineStr"/>
-      <c r="C28" s="206" t="inlineStr"/>
-      <c r="D28" s="202" t="inlineStr">
+      <c r="A28" s="201" t="inlineStr"/>
+      <c r="B28" s="201" t="inlineStr"/>
+      <c r="C28" s="201" t="inlineStr"/>
+      <c r="D28" s="197" t="inlineStr">
         <is>
           <t>الأدنى (Low) — قبل Q1</t>
         </is>
       </c>
-      <c r="E28" s="203" t="n">
+      <c r="E28" s="198" t="n">
         <v>80</v>
       </c>
-      <c r="F28" s="204" t="inlineStr">
+      <c r="F28" s="199" t="inlineStr">
         <is>
           <t>شراء</t>
         </is>
       </c>
-      <c r="G28" s="205" t="inlineStr">
-        <is>
-          <t>+110.5%</t>
+      <c r="G28" s="200" t="inlineStr">
+        <is>
+          <t>+5.4%</t>
         </is>
       </c>
     </row>
@@ -10135,81 +10117,81 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="180" t="inlineStr">
+      <c r="A30" s="177" t="inlineStr">
         <is>
           <t>اكسترا</t>
         </is>
       </c>
-      <c r="B30" s="181" t="inlineStr">
+      <c r="B30" s="178" t="inlineStr">
         <is>
           <t>4003</t>
         </is>
       </c>
-      <c r="C30" s="182" t="n">
-        <v>95</v>
-      </c>
-      <c r="D30" s="183" t="inlineStr">
+      <c r="C30" s="179" t="n">
+        <v>81.90000000000001</v>
+      </c>
+      <c r="D30" s="180" t="inlineStr">
         <is>
           <t>إجماع (8 محللين)</t>
         </is>
       </c>
-      <c r="E30" s="188" t="n">
+      <c r="E30" s="181" t="n">
         <v>111.7</v>
       </c>
-      <c r="F30" s="185" t="inlineStr">
+      <c r="F30" s="182" t="inlineStr">
         <is>
           <t>شراء قوي (Strong Buy)</t>
         </is>
       </c>
-      <c r="G30" s="189" t="inlineStr">
-        <is>
-          <t>+17.6%</t>
+      <c r="G30" s="183" t="inlineStr">
+        <is>
+          <t>+36.4%</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="187" t="inlineStr"/>
-      <c r="B31" s="187" t="inlineStr"/>
-      <c r="C31" s="187" t="inlineStr"/>
-      <c r="D31" s="183" t="inlineStr">
+      <c r="A31" s="184" t="inlineStr"/>
+      <c r="B31" s="184" t="inlineStr"/>
+      <c r="C31" s="184" t="inlineStr"/>
+      <c r="D31" s="180" t="inlineStr">
         <is>
           <t>الأعلى (High)</t>
         </is>
       </c>
-      <c r="E31" s="188" t="n">
+      <c r="E31" s="181" t="n">
         <v>140</v>
       </c>
-      <c r="F31" s="185" t="inlineStr">
+      <c r="F31" s="182" t="inlineStr">
         <is>
           <t>شراء قوي</t>
         </is>
       </c>
-      <c r="G31" s="189" t="inlineStr">
-        <is>
-          <t>+47.4%</t>
+      <c r="G31" s="183" t="inlineStr">
+        <is>
+          <t>+70.9%</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="187" t="inlineStr"/>
-      <c r="B32" s="187" t="inlineStr"/>
-      <c r="C32" s="187" t="inlineStr"/>
-      <c r="D32" s="183" t="inlineStr">
+      <c r="A32" s="184" t="inlineStr"/>
+      <c r="B32" s="184" t="inlineStr"/>
+      <c r="C32" s="184" t="inlineStr"/>
+      <c r="D32" s="180" t="inlineStr">
         <is>
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E32" s="184" t="n">
+      <c r="E32" s="181" t="n">
         <v>93</v>
       </c>
-      <c r="F32" s="185" t="inlineStr">
+      <c r="F32" s="182" t="inlineStr">
         <is>
           <t>شراء</t>
         </is>
       </c>
-      <c r="G32" s="186" t="inlineStr">
-        <is>
-          <t>-2.1%</t>
+      <c r="G32" s="183" t="inlineStr">
+        <is>
+          <t>+13.6%</t>
         </is>
       </c>
     </row>
@@ -10226,76 +10208,76 @@
           <t>المتقدمة</t>
         </is>
       </c>
-      <c r="B34" s="207" t="inlineStr">
+      <c r="B34" s="202" t="inlineStr">
         <is>
           <t>2330</t>
         </is>
       </c>
       <c r="C34" s="120" t="n">
-        <v>48</v>
-      </c>
-      <c r="D34" s="208" t="inlineStr">
+        <v>30</v>
+      </c>
+      <c r="D34" s="203" t="inlineStr">
         <is>
           <t>إجماع (8 محللين)</t>
         </is>
       </c>
-      <c r="E34" s="209" t="n">
+      <c r="E34" s="204" t="n">
         <v>38.8</v>
       </c>
-      <c r="F34" s="210" t="inlineStr">
+      <c r="F34" s="205" t="inlineStr">
         <is>
           <t>محايد (Hold)</t>
         </is>
       </c>
-      <c r="G34" s="211" t="inlineStr">
-        <is>
-          <t>-19.2%</t>
+      <c r="G34" s="127" t="inlineStr">
+        <is>
+          <t>+29.3%</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="212" t="inlineStr"/>
-      <c r="B35" s="212" t="inlineStr"/>
-      <c r="C35" s="212" t="inlineStr"/>
-      <c r="D35" s="208" t="inlineStr">
+      <c r="A35" s="206" t="inlineStr"/>
+      <c r="B35" s="206" t="inlineStr"/>
+      <c r="C35" s="206" t="inlineStr"/>
+      <c r="D35" s="203" t="inlineStr">
         <is>
           <t>الأعلى (High)</t>
         </is>
       </c>
-      <c r="E35" s="213" t="n">
+      <c r="E35" s="204" t="n">
         <v>50</v>
       </c>
-      <c r="F35" s="210" t="inlineStr">
+      <c r="F35" s="205" t="inlineStr">
         <is>
           <t>شراء — عند التعافي</t>
         </is>
       </c>
       <c r="G35" s="127" t="inlineStr">
         <is>
-          <t>+4.2%</t>
+          <t>+66.7%</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="212" t="inlineStr"/>
-      <c r="B36" s="212" t="inlineStr"/>
-      <c r="C36" s="212" t="inlineStr"/>
-      <c r="D36" s="208" t="inlineStr">
+      <c r="A36" s="206" t="inlineStr"/>
+      <c r="B36" s="206" t="inlineStr"/>
+      <c r="C36" s="206" t="inlineStr"/>
+      <c r="D36" s="203" t="inlineStr">
         <is>
           <t>الأدنى (Low)</t>
         </is>
       </c>
-      <c r="E36" s="209" t="n">
+      <c r="E36" s="204" t="n">
         <v>31.1</v>
       </c>
-      <c r="F36" s="210" t="inlineStr">
+      <c r="F36" s="205" t="inlineStr">
         <is>
           <t>بيع / تخفيض</t>
         </is>
       </c>
-      <c r="G36" s="211" t="inlineStr">
-        <is>
-          <t>-35.2%</t>
+      <c r="G36" s="207" t="inlineStr">
+        <is>
+          <t>+3.7%</t>
         </is>
       </c>
     </row>
@@ -10307,30 +10289,30 @@
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="147" t="inlineStr">
+      <c r="A38" s="146" t="inlineStr">
         <is>
           <t>بنيان ريت</t>
         </is>
       </c>
-      <c r="B38" s="214" t="inlineStr">
+      <c r="B38" s="208" t="inlineStr">
         <is>
           <t>4340</t>
         </is>
       </c>
-      <c r="C38" s="148" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="D38" s="215" t="inlineStr">
+      <c r="C38" s="147" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="D38" s="209" t="inlineStr">
         <is>
           <t>لا تغطية موثقة من بيوت خبرة</t>
         </is>
       </c>
-      <c r="E38" s="216" t="inlineStr">
+      <c r="E38" s="210" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F38" s="217" t="inlineStr">
+      <c r="F38" s="211" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -10349,7 +10331,7 @@
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="218" t="inlineStr">
+      <c r="A41" s="212" t="inlineStr">
         <is>
           <t>🟢 Upside &gt; +5%  =  فرصة رأسمالية   |   🟡 بين ±5%  =  تقييم عادل   |   🔴 Downside &gt; -5%  =  مكلف أو بلغ هدفه</t>
         </is>
@@ -10436,12 +10418,12 @@
           <t>الراجحي</t>
         </is>
       </c>
-      <c r="B3" s="219" t="inlineStr">
+      <c r="B3" s="213" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
-      <c r="C3" s="155" t="inlineStr">
+      <c r="C3" s="154" t="inlineStr">
         <is>
           <t>18%</t>
         </is>
@@ -10451,12 +10433,12 @@
           <t>18,000 ريال</t>
         </is>
       </c>
-      <c r="E3" s="220" t="inlineStr">
+      <c r="E3" s="214" t="inlineStr">
         <is>
           <t>نواة البنوك الإسلامية · توزيعات مستقرة · رؤية 2030</t>
         </is>
       </c>
-      <c r="F3" s="221" t="inlineStr">
+      <c r="F3" s="215" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
@@ -10468,12 +10450,12 @@
           <t>STC</t>
         </is>
       </c>
-      <c r="B4" s="219" t="inlineStr">
+      <c r="B4" s="213" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
-      <c r="C4" s="155" t="inlineStr">
+      <c r="C4" s="154" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
@@ -10483,12 +10465,12 @@
           <t>15,000 ريال</t>
         </is>
       </c>
-      <c r="E4" s="220" t="inlineStr">
+      <c r="E4" s="214" t="inlineStr">
         <is>
           <t>أعلى عائد توزيع · البنية الرقمية الوطنية</t>
         </is>
       </c>
-      <c r="F4" s="155" t="inlineStr">
+      <c r="F4" s="154" t="inlineStr">
         <is>
           <t>منخفض</t>
         </is>
@@ -10500,12 +10482,12 @@
           <t>اكسترا</t>
         </is>
       </c>
-      <c r="B5" s="222" t="inlineStr">
+      <c r="B5" s="216" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C5" s="223" t="inlineStr">
+      <c r="C5" s="217" t="inlineStr">
         <is>
           <t>12%</t>
         </is>
@@ -10515,12 +10497,12 @@
           <t>12,000 ريال</t>
         </is>
       </c>
-      <c r="E5" s="224" t="inlineStr">
+      <c r="E5" s="218" t="inlineStr">
         <is>
           <t>قطاع التجزئة الدفاعي · توزيعات ممتازة · هامش أمان جيد</t>
         </is>
       </c>
-      <c r="F5" s="225" t="inlineStr">
+      <c r="F5" s="219" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
@@ -10532,12 +10514,12 @@
           <t>المواساة</t>
         </is>
       </c>
-      <c r="B6" s="222" t="inlineStr">
+      <c r="B6" s="216" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C6" s="223" t="inlineStr">
+      <c r="C6" s="217" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
@@ -10547,12 +10529,12 @@
           <t>10,000 ريال</t>
         </is>
       </c>
-      <c r="E6" s="224" t="inlineStr">
+      <c r="E6" s="218" t="inlineStr">
         <is>
           <t>رعاية صحية دفاعية · توزيع سنوي منتظم</t>
         </is>
       </c>
-      <c r="F6" s="223" t="inlineStr">
+      <c r="F6" s="217" t="inlineStr">
         <is>
           <t>منخفض</t>
         </is>
@@ -10564,12 +10546,12 @@
           <t>الإنماء</t>
         </is>
       </c>
-      <c r="B7" s="226" t="inlineStr">
+      <c r="B7" s="220" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
-      <c r="C7" s="227" t="inlineStr">
+      <c r="C7" s="221" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
@@ -10579,12 +10561,12 @@
           <t>10,000 ريال</t>
         </is>
       </c>
-      <c r="E7" s="228" t="inlineStr">
+      <c r="E7" s="222" t="inlineStr">
         <is>
           <t>أسرع البنوك نمواً · تراجع تقييم يوفر دخولاً جيدة</t>
         </is>
       </c>
-      <c r="F7" s="229" t="inlineStr">
+      <c r="F7" s="223" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
@@ -10596,12 +10578,12 @@
           <t>سال</t>
         </is>
       </c>
-      <c r="B8" s="226" t="inlineStr">
+      <c r="B8" s="220" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
-      <c r="C8" s="230" t="inlineStr">
+      <c r="C8" s="224" t="inlineStr">
         <is>
           <t>7%</t>
         </is>
@@ -10611,12 +10593,12 @@
           <t>7,000 ريال</t>
         </is>
       </c>
-      <c r="E8" s="228" t="inlineStr">
+      <c r="E8" s="222" t="inlineStr">
         <is>
           <t>الاستفادة من نمو قطاع الخدمات اللوجستية الجوية</t>
         </is>
       </c>
-      <c r="F8" s="231" t="inlineStr">
+      <c r="F8" s="225" t="inlineStr">
         <is>
           <t>متوسط</t>
         </is>
@@ -10628,12 +10610,12 @@
           <t>بنيان ريت</t>
         </is>
       </c>
-      <c r="B9" s="222" t="inlineStr">
+      <c r="B9" s="216" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C9" s="232" t="inlineStr">
+      <c r="C9" s="226" t="inlineStr">
         <is>
           <t>8%</t>
         </is>
@@ -10643,12 +10625,12 @@
           <t>8,000 ريال</t>
         </is>
       </c>
-      <c r="E9" s="224" t="inlineStr">
+      <c r="E9" s="218" t="inlineStr">
         <is>
           <t>دخل إيجاري ثابت · عائد توزيع مرتفع · تنويع القطاعات</t>
         </is>
       </c>
-      <c r="F9" s="225" t="inlineStr">
+      <c r="F9" s="219" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
@@ -10660,12 +10642,12 @@
           <t>المتقدمة</t>
         </is>
       </c>
-      <c r="B10" s="219" t="inlineStr">
+      <c r="B10" s="213" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
-      <c r="C10" s="233" t="inlineStr">
+      <c r="C10" s="227" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
@@ -10675,83 +10657,83 @@
           <t>5,000 ريال</t>
         </is>
       </c>
-      <c r="E10" s="220" t="inlineStr">
+      <c r="E10" s="214" t="inlineStr">
         <is>
           <t>وزن محدود · مضاربة على العودة للربحية + رؤية 2030</t>
         </is>
       </c>
-      <c r="F10" s="234" t="inlineStr">
+      <c r="F10" s="228" t="inlineStr">
         <is>
           <t>مرتفع</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="235" t="inlineStr">
+      <c r="A11" s="229" t="inlineStr">
         <is>
           <t>بدجت</t>
         </is>
       </c>
-      <c r="B11" s="236" t="inlineStr">
+      <c r="B11" s="230" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
-      <c r="C11" s="237" t="inlineStr">
+      <c r="C11" s="231" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="D11" s="238" t="inlineStr">
+      <c r="D11" s="232" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="239" t="inlineStr">
+      <c r="E11" s="233" t="inlineStr">
         <is>
           <t>⚠ تأجيل حتى توضيح أسباب تراجع Q1 2026</t>
         </is>
       </c>
-      <c r="F11" s="240" t="inlineStr">
+      <c r="F11" s="234" t="inlineStr">
         <is>
           <t>متوسط-مرتفع</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="241" t="inlineStr">
+      <c r="A12" s="235" t="inlineStr">
         <is>
           <t>كاش</t>
         </is>
       </c>
-      <c r="B12" s="242" t="inlineStr">
+      <c r="B12" s="236" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C12" s="243" t="inlineStr">
+      <c r="C12" s="237" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="D12" s="244" t="inlineStr">
+      <c r="D12" s="238" t="inlineStr">
         <is>
           <t>15,000 ريال</t>
         </is>
       </c>
-      <c r="E12" s="245" t="inlineStr">
+      <c r="E12" s="239" t="inlineStr">
         <is>
           <t>احتياطي للشراء عند الانخفاض · الحد الأدنى المقترح</t>
         </is>
       </c>
-      <c r="F12" s="246" t="inlineStr">
+      <c r="F12" s="240" t="inlineStr">
         <is>
           <t>صفر</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="247" t="inlineStr">
+      <c r="A14" s="241" t="inlineStr">
         <is>
           <t>استراتيجية الشراء التدريجي (Staggered Entry):
 • المرحلة 1 (الآن): الراجحي + STC + اكسترا + المواساة = 55% من المحفظة (على دفعتين)
@@ -10802,132 +10784,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>69.09999999999999</v>
+      <c r="B3" s="244" t="n">
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>40000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>4000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>2.76</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>3.9</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>20.2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Blend</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>تراكم</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -10954,80 +10936,80 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>23500</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>30100</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>29800</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>34200</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>14979</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>17151</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>16621</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>19722</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>12000</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>16000</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>14500</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>18500</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: تمويل مشاريع عملاقة + صيرفة إسلامية + تمويل الأفراد + رقمنة الخدمات</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: متطلبات كفاية رأس المال (SAMA) · تأثير المنح على المعدلات للسهم · تنافسية ضيقة</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
-        <is>
-          <t>⚠ تنبيه: ⚠ منح سهم لكل سهمين في H2 2025 → سترتفع الأسهم إلى 6,000M</t>
+      <c r="A22" s="253" t="inlineStr">
+        <is>
+          <t>⚠ تنبيه: ✅ سعر مُعدَّل بعد المنح (1 سهم / 2) → الأسهم ارتفعت من 4B إلى 6B</t>
         </is>
       </c>
     </row>
@@ -11068,132 +11050,132 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="248" t="inlineStr">
+      <c r="A2" s="242" t="inlineStr">
         <is>
           <t>المؤشر</t>
         </is>
       </c>
-      <c r="B2" s="248" t="inlineStr">
+      <c r="B2" s="242" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="249" t="inlineStr">
+      <c r="A3" s="243" t="inlineStr">
         <is>
           <t>السعر الحالي (ريال)</t>
         </is>
       </c>
-      <c r="B3" s="250" t="n">
-        <v>27.5</v>
+      <c r="B3" s="244" t="n">
+        <v>23.53</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="245" t="inlineStr">
         <is>
           <t>رأس المال (م.ريال)</t>
         </is>
       </c>
-      <c r="B4" s="252" t="n">
+      <c r="B4" s="246" t="n">
         <v>19922</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="249" t="inlineStr">
+      <c r="A5" s="243" t="inlineStr">
         <is>
           <t>عدد الأسهم (م.سهم)</t>
         </is>
       </c>
-      <c r="B5" s="250" t="n">
+      <c r="B5" s="244" t="n">
         <v>1992</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="245" t="inlineStr">
         <is>
           <t>مضاعف الربحية (P/E)</t>
         </is>
       </c>
-      <c r="B6" s="252" t="n">
+      <c r="B6" s="246" t="n">
         <v>9.4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="249" t="inlineStr">
+      <c r="A7" s="243" t="inlineStr">
         <is>
           <t>مضاعف الدفتري (P/B)</t>
         </is>
       </c>
-      <c r="B7" s="250" t="n">
+      <c r="B7" s="244" t="n">
         <v>1.86</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="245" t="inlineStr">
         <is>
           <t>عائد التوزيع %</t>
         </is>
       </c>
-      <c r="B8" s="252" t="n">
+      <c r="B8" s="246" t="n">
         <v>4.4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="249" t="inlineStr">
+      <c r="A9" s="243" t="inlineStr">
         <is>
           <t>العائد على حقوق المساهمين %</t>
         </is>
       </c>
-      <c r="B9" s="250" t="n">
+      <c r="B9" s="244" t="n">
         <v>21.3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="245" t="inlineStr">
         <is>
           <t>تصنيف المحفظة</t>
         </is>
       </c>
-      <c r="B10" s="252" t="inlineStr">
+      <c r="B10" s="246" t="inlineStr">
         <is>
           <t>Growth</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="249" t="inlineStr">
+      <c r="A11" s="243" t="inlineStr">
         <is>
           <t>مستوى المخاطرة</t>
         </is>
       </c>
-      <c r="B11" s="250" t="inlineStr">
+      <c r="B11" s="244" t="inlineStr">
         <is>
           <t>منخفض-متوسط</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="245" t="inlineStr">
         <is>
           <t>التوصية</t>
         </is>
       </c>
-      <c r="B12" s="252" t="inlineStr">
+      <c r="B12" s="246" t="inlineStr">
         <is>
           <t>تراكم</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="253" t="inlineStr">
+      <c r="A14" s="247" t="inlineStr">
         <is>
           <t>الأداء المالي التاريخي (مليون ريال)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="254" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>البند</t>
         </is>
@@ -11220,78 +11202,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="255" t="inlineStr">
+      <c r="A16" s="249" t="inlineStr">
         <is>
           <t>الإيرادات</t>
         </is>
       </c>
-      <c r="B16" s="256" t="n">
+      <c r="B16" s="250" t="n">
         <v>5500</v>
       </c>
-      <c r="C16" s="256" t="n">
+      <c r="C16" s="250" t="n">
         <v>7200</v>
       </c>
-      <c r="D16" s="256" t="n">
+      <c r="D16" s="250" t="n">
         <v>8700</v>
       </c>
-      <c r="E16" s="256" t="n">
+      <c r="E16" s="250" t="n">
         <v>10200</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="255" t="inlineStr">
+      <c r="A17" s="249" t="inlineStr">
         <is>
           <t>صافي الربح</t>
         </is>
       </c>
-      <c r="B17" s="256" t="n">
+      <c r="B17" s="250" t="n">
         <v>2714</v>
       </c>
-      <c r="C17" s="256" t="n">
+      <c r="C17" s="250" t="n">
         <v>3599</v>
       </c>
-      <c r="D17" s="256" t="n">
+      <c r="D17" s="250" t="n">
         <v>4839</v>
       </c>
-      <c r="E17" s="256" t="n">
+      <c r="E17" s="250" t="n">
         <v>5832</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="255" t="inlineStr">
+      <c r="A18" s="249" t="inlineStr">
         <is>
           <t>التدفق النقدي التشغيلي</t>
         </is>
       </c>
-      <c r="B18" s="256" t="n">
+      <c r="B18" s="250" t="n">
         <v>3000</v>
       </c>
-      <c r="C18" s="256" t="n">
+      <c r="C18" s="250" t="n">
         <v>4200</v>
       </c>
-      <c r="D18" s="256" t="n">
+      <c r="D18" s="250" t="n">
         <v>5500</v>
       </c>
-      <c r="E18" s="256" t="n">
+      <c r="E18" s="250" t="n">
         <v>6800</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="257" t="inlineStr">
+      <c r="A20" s="251" t="inlineStr">
         <is>
           <t>رؤية 2030 والمحفزات: تمويل المشاريع الكبرى + تمويل الرهن العقاري + SME Lending + رقمنة</t>
         </is>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="258" t="inlineStr">
+      <c r="A21" s="252" t="inlineStr">
         <is>
           <t>المخاطر: بنك أصغر نسبياً · انكشاف عقاري · سيولة تداول أقل</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="259" t="inlineStr">
+      <c r="A22" s="253" t="inlineStr">
         <is>
           <t>⚠ تنبيه: تحول إلى توزيعات ربعية منذ 2023</t>
         </is>

</xml_diff>